<commit_message>
Minor updates on inputs and visualization
</commit_message>
<xml_diff>
--- a/inputs/dma_params_new.xlsx
+++ b/inputs/dma_params_new.xlsx
@@ -1,29 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\hmdni\OneDrive\Documents\GitHub\odias\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB370A68-9D8B-4B17-9DB8-9296ADDE2040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A272E8-7BA3-429C-B478-921EE6412F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5295" yWindow="2940" windowWidth="15060" windowHeight="11295" firstSheet="3" activeTab="3" xr2:uid="{BF76CB6B-6024-45E4-967E-95DB60FBF193}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BF76CB6B-6024-45E4-967E-95DB60FBF193}"/>
   </bookViews>
   <sheets>
-    <sheet name="30JUL24_HIGHAGGLOM_TANDEM" sheetId="16" r:id="rId1"/>
-    <sheet name="26JUL24_LOWAGGLOM_TANDEM" sheetId="17" r:id="rId2"/>
-    <sheet name="28AUG24_HIGHAGGLOM_TANDEM" sheetId="15" r:id="rId3"/>
-    <sheet name="20AUG24_HIGHAGGLOM_TANDEM" sheetId="14" r:id="rId4"/>
-    <sheet name="20AUG24_LOWAGGLOM_TANDEM" sheetId="13" r:id="rId5"/>
-    <sheet name="21AUG24_HIGHAGGLOM_TANDEM" sheetId="12" r:id="rId6"/>
-    <sheet name="19AUG24_LOWAGGLOM_TANDEM" sheetId="11" r:id="rId7"/>
-    <sheet name="ET017_NIT013_AIR16_DIST" sheetId="10" r:id="rId8"/>
-    <sheet name="23JUL24_SWEEP_ON_AIR" sheetId="8" r:id="rId9"/>
-    <sheet name="20JUL24_SWEEP_ON_NITROGEN" sheetId="9" r:id="rId10"/>
-    <sheet name="13SEP24_SWEEP_ON_FUEL" sheetId="7" r:id="rId11"/>
+    <sheet name="07FEB25_EXCOLAPS_TANDEM" sheetId="20" r:id="rId1"/>
+    <sheet name="06FEB25_R2_EXAGGLOM_TANDEM" sheetId="19" r:id="rId2"/>
+    <sheet name="06FEB25_R1_EXAGGLOM_TANDEM" sheetId="18" r:id="rId3"/>
+    <sheet name="30JUL24_HIGHAGGLOM_TANDEM" sheetId="16" r:id="rId4"/>
+    <sheet name="26JUL24_LOWAGGLOM_TANDEM" sheetId="17" r:id="rId5"/>
+    <sheet name="28AUG24_HIGHAGGLOM_TANDEM" sheetId="15" r:id="rId6"/>
+    <sheet name="20AUG24_HIGHAGGLOM_TANDEM" sheetId="14" r:id="rId7"/>
+    <sheet name="20AUG24_LOWAGGLOM_TANDEM" sheetId="13" r:id="rId8"/>
+    <sheet name="21AUG24_HIGHAGGLOM_TANDEM" sheetId="12" r:id="rId9"/>
+    <sheet name="19AUG24_LOWAGGLOM_TANDEM" sheetId="11" r:id="rId10"/>
+    <sheet name="ET017_NIT013_AIR16_DIST" sheetId="10" r:id="rId11"/>
+    <sheet name="23JUL24_SWEEP_ON_AIR" sheetId="8" r:id="rId12"/>
+    <sheet name="20JUL24_SWEEP_ON_NITROGEN" sheetId="9" r:id="rId13"/>
+    <sheet name="13SEP24_SWEEP_ON_FUEL" sheetId="7" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="167">
   <si>
     <t>1:3</t>
   </si>
@@ -451,6 +454,102 @@
   </si>
   <si>
     <t>2024-07-30_203242_SMPS</t>
+  </si>
+  <si>
+    <t>D:\Hamed\CND\PhD\Experiments\PFA-RH122\PFA results\SMPS\FEB25-Final\FEB25-Final\TSI_Data\dn_MCC-_DLC-</t>
+  </si>
+  <si>
+    <t>2025-02-06_153534_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_154946_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_161211_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_162548_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_163937_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_165414_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_170904_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_173227_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_175756_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_181224_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_202316_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_203727_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_210954_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_212615_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_220141_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_221534_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_225352_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_223721_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_231213_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-06_205441_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_155847_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_162120_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_164259_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_165639_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_171017_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_172822_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_174347_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_175850_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_181821_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_184135_SMPS</t>
+  </si>
+  <si>
+    <t>2025-02-07_185531_SMPS</t>
   </si>
 </sst>
 </file>
@@ -846,6 +945,2118 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C54D949B-5926-4535-8FE9-0665F7DCA5DD}">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36.7109375" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C2" s="5">
+        <v>80</v>
+      </c>
+      <c r="D2" s="4">
+        <v>7.22</v>
+      </c>
+      <c r="E2" s="5">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" s="5">
+        <v>88.7</v>
+      </c>
+      <c r="D3" s="4">
+        <v>8.07</v>
+      </c>
+      <c r="E3" s="5">
+        <v>9</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" s="5">
+        <v>98.4</v>
+      </c>
+      <c r="D4" s="4">
+        <v>8.92</v>
+      </c>
+      <c r="E4" s="5">
+        <v>7</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C5" s="5">
+        <v>109.1</v>
+      </c>
+      <c r="D5" s="4">
+        <v>9.91</v>
+      </c>
+      <c r="E5" s="5">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C6" s="5">
+        <v>120.9</v>
+      </c>
+      <c r="D6" s="4">
+        <v>10.68</v>
+      </c>
+      <c r="E6" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C7" s="5">
+        <v>134.11108308881299</v>
+      </c>
+      <c r="D7" s="4">
+        <v>11.45</v>
+      </c>
+      <c r="E7" s="5">
+        <v>4</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C8" s="5">
+        <v>148.69999999999999</v>
+      </c>
+      <c r="D8" s="4">
+        <v>12.3</v>
+      </c>
+      <c r="E8" s="5">
+        <v>3</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C9" s="5">
+        <v>164.9</v>
+      </c>
+      <c r="D9" s="4">
+        <v>13.08</v>
+      </c>
+      <c r="E9" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C10" s="5">
+        <v>182.8</v>
+      </c>
+      <c r="D10" s="4">
+        <v>14.02</v>
+      </c>
+      <c r="E10" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C11" s="5">
+        <v>202.8</v>
+      </c>
+      <c r="D11" s="4">
+        <v>14.93</v>
+      </c>
+      <c r="E11" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>166</v>
+      </c>
+      <c r="C12" s="5">
+        <v>224.8</v>
+      </c>
+      <c r="D12" s="4">
+        <v>15</v>
+      </c>
+      <c r="E12" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>166</v>
+      </c>
+      <c r="C13" s="5">
+        <v>249.3</v>
+      </c>
+      <c r="D13" s="4">
+        <v>15</v>
+      </c>
+      <c r="E13" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G13" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C14" s="5"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E16" s="5"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E17" s="5"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54E29823-EAED-4A25-8B8F-59B6950B05BB}">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36.7109375" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="4">
+        <v>31.5</v>
+      </c>
+      <c r="D2" s="4">
+        <v>2.84</v>
+      </c>
+      <c r="E2" s="5">
+        <v>15</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="4">
+        <v>37</v>
+      </c>
+      <c r="D3" s="4">
+        <v>3.36</v>
+      </c>
+      <c r="E3" s="5">
+        <v>15</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="4">
+        <v>43.3</v>
+      </c>
+      <c r="D4" s="4">
+        <v>3.93</v>
+      </c>
+      <c r="E4" s="5">
+        <v>15</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="4">
+        <v>50.8</v>
+      </c>
+      <c r="D5" s="4">
+        <v>4.62</v>
+      </c>
+      <c r="E5" s="5">
+        <v>15</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="4">
+        <v>59.5</v>
+      </c>
+      <c r="D6" s="4">
+        <v>5.4</v>
+      </c>
+      <c r="E6" s="5">
+        <v>12</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="4">
+        <v>69.7</v>
+      </c>
+      <c r="D7" s="4">
+        <v>6.33</v>
+      </c>
+      <c r="E7" s="5">
+        <v>12</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="4">
+        <v>81.7</v>
+      </c>
+      <c r="D8" s="4">
+        <v>7.41</v>
+      </c>
+      <c r="E8" s="5">
+        <v>6</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="4">
+        <v>95.8</v>
+      </c>
+      <c r="D9" s="4">
+        <v>8.67</v>
+      </c>
+      <c r="E9" s="5">
+        <v>6</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="4">
+        <v>112.3</v>
+      </c>
+      <c r="D10" s="4">
+        <v>10.09</v>
+      </c>
+      <c r="E10" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="4">
+        <v>131.6</v>
+      </c>
+      <c r="D11" s="4">
+        <v>11.25</v>
+      </c>
+      <c r="E11" s="5">
+        <v>3</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="4">
+        <v>154.30000000000001</v>
+      </c>
+      <c r="D12" s="4">
+        <v>12.53</v>
+      </c>
+      <c r="E12" s="5">
+        <v>3</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="4">
+        <v>180.8</v>
+      </c>
+      <c r="D13" s="4">
+        <v>13.86</v>
+      </c>
+      <c r="E13" s="5">
+        <v>3</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="4">
+        <v>211.9</v>
+      </c>
+      <c r="D14" s="4">
+        <v>15</v>
+      </c>
+      <c r="E14" s="5">
+        <v>3</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E15" s="5"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E16" s="5"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E17" s="5"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05AE73DF-AC79-457F-9CE4-E6FEFB9D1C73}">
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="68.28515625" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="5">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97E1FF8C-F2C6-4468-9BAB-5FF356FF2B49}">
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="29.42578125" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="5">
+        <v>3</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E16" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A154C9C-AB65-4231-8298-10E3CEF878B7}">
+  <dimension ref="A1:H47"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="2"/>
+    <col min="5" max="5" width="9.140625" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>20</v>
+      </c>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>20</v>
+      </c>
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>20</v>
+      </c>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="C27" s="5"/>
+      <c r="E27" s="4"/>
+      <c r="F27"/>
+      <c r="G27"/>
+      <c r="H27"/>
+    </row>
+    <row r="47" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2"/>
+      <c r="B47" s="3"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="4"/>
+      <c r="F47"/>
+      <c r="G47"/>
+      <c r="H47"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E154B3E6-2BDE-4817-B65C-F71F8F992F62}">
+  <dimension ref="A1:H48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34" style="2" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="2"/>
+    <col min="5" max="5" width="9.140625" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="4">
+        <v>20</v>
+      </c>
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="4">
+        <v>20</v>
+      </c>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="4">
+        <v>20</v>
+      </c>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+    </row>
+    <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3"/>
+      <c r="C28" s="5"/>
+      <c r="E28" s="4"/>
+      <c r="F28"/>
+      <c r="G28"/>
+      <c r="H28"/>
+    </row>
+    <row r="48" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2"/>
+      <c r="B48" s="3"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="4"/>
+      <c r="F48"/>
+      <c r="G48"/>
+      <c r="H48"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04004435-AE29-4896-B73A-85B7E695DE36}">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36.7109375" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C2" s="5">
+        <v>70</v>
+      </c>
+      <c r="D2" s="4">
+        <v>6.35</v>
+      </c>
+      <c r="E2" s="5">
+        <v>9</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C3" s="5">
+        <v>78.900000000000006</v>
+      </c>
+      <c r="D3" s="4">
+        <v>7.16</v>
+      </c>
+      <c r="E3" s="5">
+        <v>7</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C4" s="5">
+        <v>89</v>
+      </c>
+      <c r="D4" s="4">
+        <v>8.08</v>
+      </c>
+      <c r="E4" s="5">
+        <v>6</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" s="5">
+        <v>100.4</v>
+      </c>
+      <c r="D5" s="4">
+        <v>9.11</v>
+      </c>
+      <c r="E5" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="5">
+        <v>113.2</v>
+      </c>
+      <c r="D6" s="4">
+        <v>10.19</v>
+      </c>
+      <c r="E6" s="5">
+        <v>3</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C7" s="5">
+        <v>127.7</v>
+      </c>
+      <c r="D7" s="4">
+        <v>11.07</v>
+      </c>
+      <c r="E7" s="5">
+        <v>3</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C8" s="5">
+        <v>144</v>
+      </c>
+      <c r="D8" s="4">
+        <v>12.01</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C9" s="5">
+        <v>162.4</v>
+      </c>
+      <c r="D9" s="4">
+        <v>13</v>
+      </c>
+      <c r="E9" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C10" s="5">
+        <v>183.1</v>
+      </c>
+      <c r="D10" s="4">
+        <v>14.01</v>
+      </c>
+      <c r="E10" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C11" s="5">
+        <v>206.5</v>
+      </c>
+      <c r="D11" s="4">
+        <v>15</v>
+      </c>
+      <c r="E11" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G11" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C12" s="5"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C13" s="5"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C14" s="5"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E16" s="5"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E17" s="5"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D1F831A-AC8F-4D5B-BE15-609F91DCBD1B}">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36.7109375" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C2" s="5">
+        <v>74.3</v>
+      </c>
+      <c r="D2" s="4">
+        <v>6.72</v>
+      </c>
+      <c r="E2" s="5">
+        <v>9</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C3" s="5">
+        <v>83.8</v>
+      </c>
+      <c r="D3" s="4">
+        <v>7.58</v>
+      </c>
+      <c r="E3" s="5">
+        <v>7</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C4" s="5">
+        <v>94.5</v>
+      </c>
+      <c r="D4" s="4">
+        <v>8.5500000000000007</v>
+      </c>
+      <c r="E4" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" s="5">
+        <v>106.6</v>
+      </c>
+      <c r="D5" s="4">
+        <v>9.6300000000000008</v>
+      </c>
+      <c r="E5" s="5">
+        <v>3</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="5">
+        <v>120.2</v>
+      </c>
+      <c r="D6" s="4">
+        <v>10.59</v>
+      </c>
+      <c r="E6" s="5">
+        <v>3</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="5">
+        <v>135.6</v>
+      </c>
+      <c r="D7" s="4">
+        <v>11.52</v>
+      </c>
+      <c r="E7" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C8" s="5">
+        <v>152.9</v>
+      </c>
+      <c r="D8" s="4">
+        <v>12.48</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C9" s="5">
+        <v>172.4</v>
+      </c>
+      <c r="D9" s="4">
+        <v>13.48</v>
+      </c>
+      <c r="E9" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C10" s="5">
+        <v>194.5</v>
+      </c>
+      <c r="D10" s="4">
+        <v>14.52</v>
+      </c>
+      <c r="E10" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C11" s="5">
+        <v>219.3</v>
+      </c>
+      <c r="D11" s="4">
+        <v>15</v>
+      </c>
+      <c r="E11" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C12" s="5"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C13" s="5"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C14" s="5"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E16" s="5"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E17" s="5"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8233F0CA-20B3-4732-AA6F-4B7FCD80809C}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1172,352 +3383,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A154C9C-AB65-4231-8298-10E3CEF878B7}">
-  <dimension ref="A1:H47"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="25.7109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="29.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="2"/>
-    <col min="5" max="5" width="9.140625" style="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="4">
-        <v>20</v>
-      </c>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="4">
-        <v>20</v>
-      </c>
-      <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4">
-        <v>20</v>
-      </c>
-      <c r="H5" s="6"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="3"/>
-    </row>
-    <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="3"/>
-      <c r="C27" s="5"/>
-      <c r="E27" s="4"/>
-      <c r="F27"/>
-      <c r="G27"/>
-      <c r="H27"/>
-    </row>
-    <row r="47" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="2"/>
-      <c r="B47" s="3"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="4"/>
-      <c r="F47"/>
-      <c r="G47"/>
-      <c r="H47"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E154B3E6-2BDE-4817-B65C-F71F8F992F62}">
-  <dimension ref="A1:H48"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="34" style="2" customWidth="1"/>
-    <col min="2" max="2" width="29.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="2"/>
-    <col min="5" max="5" width="9.140625" style="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="4">
-        <v>20</v>
-      </c>
-      <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="4">
-        <v>20</v>
-      </c>
-      <c r="H4" s="1"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="4">
-        <v>20</v>
-      </c>
-      <c r="H6" s="6"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="3"/>
-    </row>
-    <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="3"/>
-      <c r="C28" s="5"/>
-      <c r="E28" s="4"/>
-      <c r="F28"/>
-      <c r="G28"/>
-      <c r="H28"/>
-    </row>
-    <row r="48" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="2"/>
-      <c r="B48" s="3"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="4"/>
-      <c r="F48"/>
-      <c r="G48"/>
-      <c r="H48"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1958237C-418B-4AB5-B19A-C844DAB948B2}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1831,7 +3697,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B63FA515-45AB-4F1C-B70B-0743E7EC282B}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2159,7 +4025,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58F64623-3178-4362-8C41-1BB89F188493}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2487,7 +4353,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7134B202-133D-4D36-B1A1-AEF7B5799E6E}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2829,7 +4695,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A3CABC4-22F8-4985-BD02-8B40F124ED82}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3154,878 +5020,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54E29823-EAED-4A25-8B8F-59B6950B05BB}">
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="36.7109375" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" s="4">
-        <v>31.5</v>
-      </c>
-      <c r="D2" s="4">
-        <v>2.84</v>
-      </c>
-      <c r="E2" s="5">
-        <v>15</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G2" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C3" s="4">
-        <v>37</v>
-      </c>
-      <c r="D3" s="4">
-        <v>3.36</v>
-      </c>
-      <c r="E3" s="5">
-        <v>15</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C4" s="4">
-        <v>43.3</v>
-      </c>
-      <c r="D4" s="4">
-        <v>3.93</v>
-      </c>
-      <c r="E4" s="5">
-        <v>15</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5" s="4">
-        <v>50.8</v>
-      </c>
-      <c r="D5" s="4">
-        <v>4.62</v>
-      </c>
-      <c r="E5" s="5">
-        <v>15</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C6" s="4">
-        <v>59.5</v>
-      </c>
-      <c r="D6" s="4">
-        <v>5.4</v>
-      </c>
-      <c r="E6" s="5">
-        <v>12</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G6" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="4">
-        <v>69.7</v>
-      </c>
-      <c r="D7" s="4">
-        <v>6.33</v>
-      </c>
-      <c r="E7" s="5">
-        <v>12</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G7" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="4">
-        <v>81.7</v>
-      </c>
-      <c r="D8" s="4">
-        <v>7.41</v>
-      </c>
-      <c r="E8" s="5">
-        <v>6</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G8" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="4">
-        <v>95.8</v>
-      </c>
-      <c r="D9" s="4">
-        <v>8.67</v>
-      </c>
-      <c r="E9" s="5">
-        <v>6</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G9" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" s="4">
-        <v>112.3</v>
-      </c>
-      <c r="D10" s="4">
-        <v>10.09</v>
-      </c>
-      <c r="E10" s="5">
-        <v>4.5</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G10" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" s="4">
-        <v>131.6</v>
-      </c>
-      <c r="D11" s="4">
-        <v>11.25</v>
-      </c>
-      <c r="E11" s="5">
-        <v>3</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G11" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="4">
-        <v>154.30000000000001</v>
-      </c>
-      <c r="D12" s="4">
-        <v>12.53</v>
-      </c>
-      <c r="E12" s="5">
-        <v>3</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G12" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" s="4">
-        <v>180.8</v>
-      </c>
-      <c r="D13" s="4">
-        <v>13.86</v>
-      </c>
-      <c r="E13" s="5">
-        <v>3</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G13" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" s="4">
-        <v>211.9</v>
-      </c>
-      <c r="D14" s="4">
-        <v>15</v>
-      </c>
-      <c r="E14" s="5">
-        <v>3</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G14" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E15" s="5"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="4"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E16" s="5"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="5:7" x14ac:dyDescent="0.25">
-      <c r="E17" s="5"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="4"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05AE73DF-AC79-457F-9CE4-E6FEFB9D1C73}">
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="68.28515625" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="5">
-        <v>3</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C6" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E11" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>50</v>
-      </c>
-      <c r="C12" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E12" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E13" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>52</v>
-      </c>
-      <c r="C14" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E14" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E15" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E16" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E17" s="4">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97E1FF8C-F2C6-4468-9BAB-5FF356FF2B49}">
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="29.42578125" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="5">
-        <v>4.5</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E11" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" s="5">
-        <v>3</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E12" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E13" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E14" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C15" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E15" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="5">
-        <v>4.5</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E16" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E17" s="4">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Added comparison of inversion methods
</commit_message>
<xml_diff>
--- a/inputs/dma_params_new.xlsx
+++ b/inputs/dma_params_new.xlsx
@@ -1,37 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\hmdni\OneDrive\Documents\GitHub\odias\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E12C7D-4118-4DBA-8571-7D0A30EBF186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C958A7-911D-4C46-A7DE-EC89D73AA95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2115" yWindow="2115" windowWidth="21600" windowHeight="11295" xr2:uid="{BF76CB6B-6024-45E4-967E-95DB60FBF193}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BF76CB6B-6024-45E4-967E-95DB60FBF193}"/>
   </bookViews>
   <sheets>
-    <sheet name="MOBIL_DIST_FEB25" sheetId="27" r:id="rId1"/>
-    <sheet name="12FEB25_R2_EXAGLOM_TANDEM" sheetId="24" r:id="rId2"/>
-    <sheet name="12FEB25_R1_EXAGLOM_TANDEM" sheetId="23" r:id="rId3"/>
-    <sheet name="11FEB25_LOAGLOM_TANDEM" sheetId="22" r:id="rId4"/>
-    <sheet name="08FEB25_EXCOLAPS_TANDEM" sheetId="21" r:id="rId5"/>
-    <sheet name="07FEB25_EXCOLAPS_TANDEM" sheetId="20" r:id="rId6"/>
-    <sheet name="06FEB25_R2_EXAGGLOM_TANDEM" sheetId="19" r:id="rId7"/>
-    <sheet name="06FEB25_R1_EXAGGLOM_TANDEM" sheetId="18" r:id="rId8"/>
-    <sheet name="30JUL24_HIGHAGGLOM_TANDEM" sheetId="16" r:id="rId9"/>
-    <sheet name="26JUL24_LOWAGGLOM_TANDEM" sheetId="17" r:id="rId10"/>
-    <sheet name="28AUG24_HIGHAGGLOM_TANDEM" sheetId="15" r:id="rId11"/>
-    <sheet name="20AUG24_HIGHAGGLOM_TANDEM" sheetId="14" r:id="rId12"/>
-    <sheet name="20AUG24_LOWAGGLOM_TANDEM" sheetId="13" r:id="rId13"/>
-    <sheet name="21AUG24_HIGHAGGLOM_TANDEM" sheetId="12" r:id="rId14"/>
-    <sheet name="19AUG24_LOWAGGLOM_TANDEM" sheetId="11" r:id="rId15"/>
-    <sheet name="ET017_NIT013_AIR16_DIST" sheetId="10" r:id="rId16"/>
-    <sheet name="23JUL24_SWEEP_ON_AIR" sheetId="8" r:id="rId17"/>
-    <sheet name="20JUL24_SWEEP_ON_NITROGEN" sheetId="9" r:id="rId18"/>
-    <sheet name="13SEP24_SWEEP_ON_FUEL" sheetId="7" r:id="rId19"/>
+    <sheet name="MAY25_TANDEM_COMPARE" sheetId="28" r:id="rId1"/>
+    <sheet name="MOBIL_DIST_FEB25" sheetId="27" r:id="rId2"/>
+    <sheet name="12FEB25_R2_EXAGLOM_TANDEM" sheetId="24" r:id="rId3"/>
+    <sheet name="12FEB25_R1_EXAGLOM_TANDEM" sheetId="23" r:id="rId4"/>
+    <sheet name="11FEB25_LOAGLOM_TANDEM" sheetId="22" r:id="rId5"/>
+    <sheet name="08FEB25_EXCOLAPS_TANDEM" sheetId="21" r:id="rId6"/>
+    <sheet name="07FEB25_EXCOLAPS_TANDEM" sheetId="20" r:id="rId7"/>
+    <sheet name="06FEB25_R2_EXAGGLOM_TANDEM" sheetId="19" r:id="rId8"/>
+    <sheet name="06FEB25_R1_EXAGGLOM_TANDEM" sheetId="18" r:id="rId9"/>
+    <sheet name="30JUL24_HIGHAGGLOM_TANDEM" sheetId="16" r:id="rId10"/>
+    <sheet name="26JUL24_LOWAGGLOM_TANDEM" sheetId="17" r:id="rId11"/>
+    <sheet name="28AUG24_HIGHAGGLOM_TANDEM" sheetId="15" r:id="rId12"/>
+    <sheet name="20AUG24_HIGHAGGLOM_TANDEM" sheetId="14" r:id="rId13"/>
+    <sheet name="20AUG24_LOWAGGLOM_TANDEM" sheetId="13" r:id="rId14"/>
+    <sheet name="21AUG24_HIGHAGGLOM_TANDEM" sheetId="12" r:id="rId15"/>
+    <sheet name="19AUG24_LOWAGGLOM_TANDEM" sheetId="11" r:id="rId16"/>
+    <sheet name="ET017_NIT013_AIR16_DIST" sheetId="10" r:id="rId17"/>
+    <sheet name="23JUL24_SWEEP_ON_AIR" sheetId="8" r:id="rId18"/>
+    <sheet name="20JUL24_SWEEP_ON_NITROGEN" sheetId="9" r:id="rId19"/>
+    <sheet name="13SEP24_SWEEP_ON_FUEL" sheetId="7" r:id="rId20"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="225">
   <si>
     <t>1:3</t>
   </si>
@@ -759,7 +760,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -778,6 +779,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -791,7 +804,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="3"/>
@@ -811,6 +824,13 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1144,270 +1164,334 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35B83332-148F-435D-8E1B-B29859C7035C}">
-  <dimension ref="A1:E22"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25DA0C63-14A2-43B6-8AB4-928023A06141}">
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.5703125" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" width="57.5703125" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="19" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="16">
+        <v>103.7</v>
+      </c>
+      <c r="D2" s="17">
+        <v>9.36</v>
+      </c>
+      <c r="E2" s="16">
+        <v>4.5</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="17">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="15"/>
+      <c r="B3" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="16">
+        <v>142.5</v>
+      </c>
+      <c r="D3" s="17">
+        <v>11.89</v>
+      </c>
+      <c r="E3" s="16">
+        <v>3</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="G3" s="17">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="15"/>
+      <c r="B4" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="17">
+        <v>180.8</v>
+      </c>
+      <c r="D4" s="17">
+        <v>13.86</v>
+      </c>
+      <c r="E4" s="16">
+        <v>3</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" s="17">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="19"/>
+      <c r="B5" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="C5" s="20">
+        <v>103.7</v>
+      </c>
+      <c r="D5" s="21">
+        <v>9.36</v>
+      </c>
+      <c r="E5" s="20">
+        <v>6</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="G5" s="21">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="19"/>
+      <c r="B6" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="C6" s="20">
+        <v>142.5</v>
+      </c>
+      <c r="D6" s="21">
+        <v>11.89</v>
+      </c>
+      <c r="E6" s="20">
+        <v>3</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="21">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="19"/>
+      <c r="B7" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="21">
+        <v>180.8</v>
+      </c>
+      <c r="D7" s="21">
+        <v>13.87</v>
+      </c>
+      <c r="E7" s="20">
+        <v>3</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="21">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="C2" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="C3" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="C4" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" s="9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="C5" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="C6" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E6" s="9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11" t="s">
-        <v>219</v>
-      </c>
-      <c r="C7" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="13">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="C8" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="9">
+      <c r="B8" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="C8" s="16">
+        <v>100.4</v>
+      </c>
+      <c r="D8" s="17">
+        <v>9.11</v>
+      </c>
+      <c r="E8" s="16">
+        <v>4.5</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="17">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="C9" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="15"/>
+      <c r="B9" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="C9" s="16">
+        <v>144</v>
+      </c>
+      <c r="D9" s="17">
+        <v>12.01</v>
+      </c>
+      <c r="E9" s="16">
+        <v>2.5</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="17">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="C10" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="9">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="C10" s="16">
+        <v>183.1</v>
+      </c>
+      <c r="D10" s="17">
+        <v>14.01</v>
+      </c>
+      <c r="E10" s="16">
+        <v>2.5</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10" s="17">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="C11" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11" t="s">
-        <v>216</v>
-      </c>
-      <c r="C12" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="E12" s="13">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="19"/>
+      <c r="B11" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="C11" s="20">
+        <v>98.4</v>
+      </c>
+      <c r="D11" s="21">
+        <v>8.92</v>
+      </c>
+      <c r="E11" s="20">
+        <v>7</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11" s="21">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="C13" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="E13" s="13">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="19"/>
+      <c r="B12" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="C12" s="20">
+        <v>141.19999999999999</v>
+      </c>
+      <c r="D12" s="21">
+        <v>11.78</v>
+      </c>
+      <c r="E12" s="20">
+        <v>3</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12" s="21">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="C14" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="E14" s="13">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="19"/>
+      <c r="B13" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="C13" s="20">
+        <v>182.8</v>
+      </c>
+      <c r="D13" s="21">
+        <v>14.02</v>
+      </c>
+      <c r="E13" s="20">
+        <v>2.5</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="G13" s="21">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="5"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="4"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D15" s="4"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="5"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="4"/>
-    </row>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D16" s="4"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
       <c r="C17" s="5"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="4"/>
-    </row>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C18" s="5"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="4"/>
-    </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C19" s="5"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="4"/>
-    </row>
-    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C20" s="5"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="4"/>
-    </row>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C21" s="5"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="4"/>
-    </row>
-    <row r="22" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C22" s="5"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G19" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1415,6 +1499,333 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8233F0CA-20B3-4732-AA6F-4B7FCD80809C}">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36.7109375" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2">
+        <v>43.3</v>
+      </c>
+      <c r="D2">
+        <v>3.93</v>
+      </c>
+      <c r="E2">
+        <v>15</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3">
+        <v>50.8</v>
+      </c>
+      <c r="D3">
+        <v>4.63</v>
+      </c>
+      <c r="E3">
+        <v>15</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4">
+        <v>59.5</v>
+      </c>
+      <c r="D4">
+        <v>5.42</v>
+      </c>
+      <c r="E4">
+        <v>15</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C5">
+        <v>69.7</v>
+      </c>
+      <c r="D5">
+        <v>6.31</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C6">
+        <v>81.7</v>
+      </c>
+      <c r="D6">
+        <v>7.39</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C7">
+        <v>95.8</v>
+      </c>
+      <c r="D7">
+        <v>8.66</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C8">
+        <v>112.3</v>
+      </c>
+      <c r="D8">
+        <v>10.07</v>
+      </c>
+      <c r="E8">
+        <v>4</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C9">
+        <v>131.6</v>
+      </c>
+      <c r="D9">
+        <v>11.27</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10">
+        <v>154.30000000000001</v>
+      </c>
+      <c r="D10">
+        <v>12.53</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C11">
+        <v>180.8</v>
+      </c>
+      <c r="D11">
+        <v>13.87</v>
+      </c>
+      <c r="E11">
+        <v>2.5</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C12">
+        <v>211.9</v>
+      </c>
+      <c r="D12">
+        <v>15</v>
+      </c>
+      <c r="E12">
+        <v>2.5</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C13">
+        <v>248.4</v>
+      </c>
+      <c r="D13">
+        <v>15</v>
+      </c>
+      <c r="E13">
+        <v>2.5</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>132</v>
+      </c>
+      <c r="C14">
+        <v>291.2</v>
+      </c>
+      <c r="D14">
+        <v>15</v>
+      </c>
+      <c r="E14">
+        <v>2.5</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E15" s="5"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E16" s="5"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E17" s="5"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1958237C-418B-4AB5-B19A-C844DAB948B2}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1728,7 +2139,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B63FA515-45AB-4F1C-B70B-0743E7EC282B}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2056,7 +2467,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58F64623-3178-4362-8C41-1BB89F188493}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2384,7 +2795,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7134B202-133D-4D36-B1A1-AEF7B5799E6E}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2726,7 +3137,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A3CABC4-22F8-4985-BD02-8B40F124ED82}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3053,7 +3464,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54E29823-EAED-4A25-8B8F-59B6950B05BB}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3381,7 +3792,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05AE73DF-AC79-457F-9CE4-E6FEFB9D1C73}">
   <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3653,7 +4064,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97E1FF8C-F2C6-4468-9BAB-5FF356FF2B49}">
   <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3927,7 +4338,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A154C9C-AB65-4231-8298-10E3CEF878B7}">
   <dimension ref="A1:H47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4085,7 +4496,278 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35B83332-148F-435D-8E1B-B29859C7035C}">
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="38.5703125" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="C2" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C3" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="C4" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7"/>
+      <c r="B5" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="C5" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7"/>
+      <c r="B6" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="C6" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="11"/>
+      <c r="B7" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="C7" s="12">
+        <v>2.5</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="C8" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C9" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7"/>
+      <c r="B10" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="C10" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C11" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="11"/>
+      <c r="B12" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="C12" s="12">
+        <v>2.5</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="C13" s="12">
+        <v>2.5</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="11"/>
+      <c r="B14" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="C14" s="12">
+        <v>2.5</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C17" s="5"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C18" s="5"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C19" s="5"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C20" s="5"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C21" s="5"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C22" s="5"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E154B3E6-2BDE-4817-B65C-F71F8F992F62}">
   <dimension ref="A1:H48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4272,7 +4954,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DE730C2-3F81-450D-9811-67897711F5B9}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4600,7 +5282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D298E7AD-F721-4288-B102-9A426DC999A3}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4915,7 +5597,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8434DCE7-790E-448F-A6D8-F6A8BEB12AED}">
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5204,7 +5886,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B527C855-2BAF-4274-B372-71B922B9578B}">
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5459,7 +6141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C54D949B-5926-4535-8FE9-0665F7DCA5DD}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5774,7 +6456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04004435-AE29-4896-B73A-85B7E695DE36}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6063,7 +6745,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D1F831A-AC8F-4D5B-BE15-609F91DCBD1B}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6350,331 +7032,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8233F0CA-20B3-4732-AA6F-4B7FCD80809C}">
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="36.7109375" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C2">
-        <v>43.3</v>
-      </c>
-      <c r="D2">
-        <v>3.93</v>
-      </c>
-      <c r="E2">
-        <v>15</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G2" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C3">
-        <v>50.8</v>
-      </c>
-      <c r="D3">
-        <v>4.63</v>
-      </c>
-      <c r="E3">
-        <v>15</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C4">
-        <v>59.5</v>
-      </c>
-      <c r="D4">
-        <v>5.42</v>
-      </c>
-      <c r="E4">
-        <v>15</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G4" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C5">
-        <v>69.7</v>
-      </c>
-      <c r="D5">
-        <v>6.31</v>
-      </c>
-      <c r="E5">
-        <v>9</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C6">
-        <v>81.7</v>
-      </c>
-      <c r="D6">
-        <v>7.39</v>
-      </c>
-      <c r="E6">
-        <v>6</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G6" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C7">
-        <v>95.8</v>
-      </c>
-      <c r="D7">
-        <v>8.66</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G7" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C8">
-        <v>112.3</v>
-      </c>
-      <c r="D8">
-        <v>10.07</v>
-      </c>
-      <c r="E8">
-        <v>4</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G8" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="C9">
-        <v>131.6</v>
-      </c>
-      <c r="D9">
-        <v>11.27</v>
-      </c>
-      <c r="E9">
-        <v>3</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G9" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="C10">
-        <v>154.30000000000001</v>
-      </c>
-      <c r="D10">
-        <v>12.53</v>
-      </c>
-      <c r="E10">
-        <v>3</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G10" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C11">
-        <v>180.8</v>
-      </c>
-      <c r="D11">
-        <v>13.87</v>
-      </c>
-      <c r="E11">
-        <v>2.5</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G11" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>130</v>
-      </c>
-      <c r="C12">
-        <v>211.9</v>
-      </c>
-      <c r="D12">
-        <v>15</v>
-      </c>
-      <c r="E12">
-        <v>2.5</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G12" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>131</v>
-      </c>
-      <c r="C13">
-        <v>248.4</v>
-      </c>
-      <c r="D13">
-        <v>15</v>
-      </c>
-      <c r="E13">
-        <v>2.5</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G13" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>132</v>
-      </c>
-      <c r="C14">
-        <v>291.2</v>
-      </c>
-      <c r="D14">
-        <v>15</v>
-      </c>
-      <c r="E14">
-        <v>2.5</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G14" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E15" s="5"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="4"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E16" s="5"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="5:7" x14ac:dyDescent="0.25">
-      <c r="E17" s="5"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="4"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>